<commit_message>
AR Voucher working state with dataprovider(Cash,Bank and PaymentInformation details provided or blank with pop up handled) Database basic validation done for finvchmain.finvchdet,finpost and fintag
</commit_message>
<xml_diff>
--- a/src/test/resources/Finance/ArVoucher.xlsx
+++ b/src/test/resources/Finance/ArVoucher.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="6900"/>
+    <workbookView windowWidth="20490" windowHeight="7620" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="DocumentInformation" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -60,12 +60,18 @@
     <t>Hena Embroidery</t>
   </si>
   <si>
-    <t>AR/AP Voucher</t>
+    <t>AR VOUCHER</t>
   </si>
   <si>
     <t>Punjab National Bank-214</t>
   </si>
   <si>
+    <t>Remarks1</t>
+  </si>
+  <si>
+    <t>Ref1</t>
+  </si>
+  <si>
     <t>LineNo</t>
   </si>
   <si>
@@ -93,6 +99,12 @@
     <t>AdjustmentType</t>
   </si>
   <si>
+    <t>PaymentSelection</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
     <t>AARUCHI FASHIONS PRIVATE LIMITED</t>
   </si>
   <si>
@@ -102,13 +114,19 @@
     <t>SelectDocument</t>
   </si>
   <si>
-    <t>ABUL KASHEM MOLLHA</t>
-  </si>
-  <si>
-    <t>J061</t>
-  </si>
-  <si>
-    <t>Sundry Creditors for Expenses</t>
+    <t>Cheque</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>AFFIFA</t>
+  </si>
+  <si>
+    <t>Sundry Debtors</t>
+  </si>
+  <si>
+    <t>NEFT/RTGS</t>
   </si>
   <si>
     <t>Payment Mode</t>
@@ -123,6 +141,12 @@
     <t>Drawn On</t>
   </si>
   <si>
+    <t>Kolkata</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
     <t>Document number</t>
   </si>
   <si>
@@ -148,9 +172,6 @@
   </si>
   <si>
     <t>VP/00754/24-25</t>
-  </si>
-  <si>
-    <t>VP/00017/25-26</t>
   </si>
   <si>
     <t>Reference Site Name</t>
@@ -167,7 +188,7 @@
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="180" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -178,6 +199,12 @@
     <font>
       <sz val="9"/>
       <color rgb="FF171D1E"/>
+      <name val="Courier New"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1F1F1F"/>
       <name val="Courier New"/>
       <charset val="134"/>
     </font>
@@ -631,164 +658,169 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -804,7 +836,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1327,16 +1359,16 @@
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="6"/>
   <cols>
-    <col min="2" max="2" width="17.7142857142857" customWidth="1"/>
-    <col min="3" max="3" width="12.2857142857143" customWidth="1"/>
-    <col min="4" max="4" width="25.8571428571429" customWidth="1"/>
-    <col min="5" max="5" width="10.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="11.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="10.8571428571429" customWidth="1"/>
+    <col min="2" max="2" width="17.7142857142857" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7142857142857" style="1" customWidth="1"/>
+    <col min="4" max="4" width="25.8571428571429" style="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5714285714286" style="1" customWidth="1"/>
+    <col min="6" max="6" width="11.1428571428571" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.8571428571429" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -1345,7 +1377,7 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
@@ -1358,8 +1390,8 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
       <c r="B2" t="s">
@@ -1371,8 +1403,14 @@
       <c r="D2" t="s">
         <v>10</v>
       </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="F2" s="5">
-        <v>46075</v>
+        <v>46121</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -1384,98 +1422,108 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2"/>
   <cols>
-    <col min="3" max="4" width="37.2857142857143" customWidth="1"/>
-    <col min="5" max="5" width="29.7142857142857" customWidth="1"/>
-    <col min="6" max="6" width="15.1428571428571" customWidth="1"/>
-    <col min="9" max="9" width="12.2857142857143" customWidth="1"/>
-    <col min="10" max="10" width="32.4285714285714" customWidth="1"/>
+    <col min="3" max="3" width="37.2857142857143" style="1" customWidth="1"/>
+    <col min="4" max="4" width="29.7142857142857" style="1" customWidth="1"/>
+    <col min="5" max="5" width="17.7142857142857" style="1" customWidth="1"/>
+    <col min="6" max="6" width="17.7142857142857" customWidth="1"/>
+    <col min="7" max="7" width="17.2857142857143" customWidth="1"/>
+    <col min="8" max="8" width="12.2857142857143" style="1" customWidth="1"/>
+    <col min="9" max="9" width="32.4285714285714" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17.4285714285714" customWidth="1"/>
+    <col min="11" max="11" width="18.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>11</v>
+      <c r="B1" t="s">
+        <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="J1" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="K1" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2">
-        <v>1</v>
+      <c r="B2" t="s">
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D2">
         <v>217</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>21</v>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
       </c>
       <c r="I2">
-        <v>200</v>
-      </c>
-      <c r="J2" t="s">
-        <v>22</v>
+        <v>2</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3" t="s">
-        <v>22</v>
+      <c r="J3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1490,38 +1538,77 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="2" width="11.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="11.4285714285714" style="1" customWidth="1"/>
+    <col min="2" max="2" width="7.85714285714286" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="16.7142857142857" customWidth="1"/>
+    <col min="6" max="6" width="10.2857142857143" customWidth="1"/>
+    <col min="7" max="7" width="10.8571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>11</v>
+      <c r="B1" t="s">
+        <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="G1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2">
+        <v>650222</v>
+      </c>
+      <c r="E2" s="5">
+        <v>46121</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="3" spans="2:2">
-      <c r="B3" s="2"/>
+    <row r="3" spans="1:7">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3">
+        <v>455352</v>
+      </c>
+      <c r="E3" s="5">
+        <v>46121</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1535,101 +1622,101 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3"/>
   <cols>
-    <col min="3" max="3" width="19.1428571428571" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="16.1428571428571" customWidth="1"/>
-    <col min="6" max="6" width="14.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="15.1428571428571" customWidth="1"/>
+    <col min="3" max="3" width="19.1428571428571" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.1428571428571" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14.1428571428571" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.1428571428571" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>11</v>
+      <c r="B1" t="s">
+        <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D1" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E1" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F1" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G1" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="H1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D2" s="4">
+      <c r="C2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="3">
         <v>45078</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>37</v>
+      <c r="E2" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="I2">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3">
         <v>1</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" s="4">
+      <c r="C3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="3">
         <v>45444</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>37</v>
+      <c r="E3" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="I3">
-        <v>199</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>39</v>
+      <c r="C4" s="2">
+        <v>270</v>
       </c>
       <c r="D4" s="4">
-        <v>46006</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>37</v>
+        <v>44783</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1644,19 +1731,19 @@
   <dimension ref="A1:C1"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="2" width="21.5714285714286" customWidth="1"/>
-    <col min="3" max="3" width="20.7142857142857" customWidth="1"/>
+    <col min="1" max="2" width="21.5714285714286" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.7142857142857" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>11</v>
+        <v>47</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ar Voucher changes where only major Select Document selection fails when document count is large like 7000 documents.Other changes has been tested and run successfully
</commit_message>
<xml_diff>
--- a/src/test/resources/Finance/ArVoucher.xlsx
+++ b/src/test/resources/Finance/ArVoucher.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" activeTab="2"/>
+    <workbookView windowWidth="20490" windowHeight="7620" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="DocumentInformation" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -105,10 +105,13 @@
     <t>1</t>
   </si>
   <si>
-    <t>AARUCHI FASHIONS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Sundry Creditors for Goods</t>
+    <t>AJEHAR  SHAIKH</t>
+  </si>
+  <si>
+    <t>J035</t>
+  </si>
+  <si>
+    <t>Sundry Creditors for Expenses</t>
   </si>
   <si>
     <t>SelectDocument</t>
@@ -117,18 +120,6 @@
     <t>Cheque</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>AFFIFA</t>
-  </si>
-  <si>
-    <t>Sundry Debtors</t>
-  </si>
-  <si>
-    <t>NEFT/RTGS</t>
-  </si>
-  <si>
     <t>Payment Mode</t>
   </si>
   <si>
@@ -141,12 +132,6 @@
     <t>Drawn On</t>
   </si>
   <si>
-    <t>Kolkata</t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-  <si>
     <t>Document number</t>
   </si>
   <si>
@@ -165,13 +150,10 @@
     <t>Adjustment Amount</t>
   </si>
   <si>
-    <t>VP/01298/23-24</t>
+    <t>VP/00275/23-24</t>
   </si>
   <si>
     <t>Voucher (AR/AP)</t>
-  </si>
-  <si>
-    <t>VP/00754/24-25</t>
   </si>
   <si>
     <t>Reference Site Name</t>
@@ -188,13 +170,19 @@
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="180" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF090909"/>
+      <name val="Segoe UI"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
@@ -205,6 +193,12 @@
     <font>
       <sz val="9"/>
       <color rgb="FF1F1F1F"/>
+      <name val="Courier New"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF0A0A0A"/>
       <name val="Courier New"/>
       <charset val="134"/>
     </font>
@@ -673,154 +667,163 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1377,7 +1380,7 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
@@ -1406,7 +1409,7 @@
       <c r="E2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="7">
         <v>46121</v>
       </c>
       <c r="G2" s="1" t="s">
@@ -1422,12 +1425,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2"/>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col min="3" max="3" width="37.2857142857143" style="1" customWidth="1"/>
     <col min="4" max="4" width="29.7142857142857" style="1" customWidth="1"/>
-    <col min="5" max="5" width="17.7142857142857" style="1" customWidth="1"/>
+    <col min="5" max="5" width="25.7142857142857" style="1" customWidth="1"/>
     <col min="6" max="6" width="17.7142857142857" customWidth="1"/>
     <col min="7" max="7" width="17.2857142857143" customWidth="1"/>
     <col min="8" max="8" width="12.2857142857143" style="1" customWidth="1"/>
@@ -1478,52 +1481,26 @@
       <c r="B2" t="s">
         <v>23</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D2">
-        <v>217</v>
+      <c r="D2" s="8" t="s">
+        <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
       </c>
       <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>26</v>
+        <v>1</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>27</v>
       </c>
       <c r="K2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
         <v>28</v>
-      </c>
-      <c r="C3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1535,8 +1512,8 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="6"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="11.4285714285714" style="1" customWidth="1"/>
     <col min="2" max="2" width="7.85714285714286" style="1" customWidth="1"/>
@@ -1555,16 +1532,16 @@
         <v>13</v>
       </c>
       <c r="C1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" t="s">
         <v>32</v>
-      </c>
-      <c r="D1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" t="s">
-        <v>35</v>
       </c>
       <c r="G1" t="s">
         <v>6</v>
@@ -1575,38 +1552,15 @@
         <v>7</v>
       </c>
       <c r="B2" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D2">
-        <v>650222</v>
-      </c>
-      <c r="E2" s="5">
-        <v>46121</v>
-      </c>
-      <c r="F2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="1">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3">
         <v>455352</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E2" s="7">
         <v>46121</v>
       </c>
     </row>
@@ -1638,25 +1592,25 @@
         <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="E1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="F1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="G1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="H1" t="s">
         <v>17</v>
       </c>
       <c r="I1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -1667,57 +1621,27 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D2" s="3">
-        <v>45078</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>45</v>
+        <v>45094</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="I2">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="3">
-        <v>45444</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="4"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4" s="2">
-        <v>270</v>
-      </c>
-      <c r="D4" s="4">
-        <v>44783</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="I4">
-        <v>2</v>
-      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1737,13 +1661,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B1" t="s">
         <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ar Voucher changes where Select Document with large no of documents pending should work along with ginesys loader handling at Select Document Opening.
</commit_message>
<xml_diff>
--- a/src/test/resources/Finance/ArVoucher.xlsx
+++ b/src/test/resources/Finance/ArVoucher.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" activeTab="3"/>
+    <workbookView windowWidth="20490" windowHeight="7620" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="DocumentInformation" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="52">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -72,6 +72,15 @@
     <t>Ref1</t>
   </si>
   <si>
+    <t>TC101</t>
+  </si>
+  <si>
+    <t>Remarks2</t>
+  </si>
+  <si>
+    <t>Ref2</t>
+  </si>
+  <si>
     <t>LineNo</t>
   </si>
   <si>
@@ -105,21 +114,27 @@
     <t>1</t>
   </si>
   <si>
-    <t>AJEHAR  SHAIKH</t>
-  </si>
-  <si>
-    <t>J035</t>
+    <t>BT CHANNEL</t>
+  </si>
+  <si>
+    <t>Sundry Debtors</t>
+  </si>
+  <si>
+    <t>SelectDocument</t>
+  </si>
+  <si>
+    <t>Cheque</t>
+  </si>
+  <si>
+    <t>ABUL KASHEM MOLLHA</t>
+  </si>
+  <si>
+    <t>J061</t>
   </si>
   <si>
     <t>Sundry Creditors for Expenses</t>
   </si>
   <si>
-    <t>SelectDocument</t>
-  </si>
-  <si>
-    <t>Cheque</t>
-  </si>
-  <si>
     <t>Payment Mode</t>
   </si>
   <si>
@@ -150,10 +165,25 @@
     <t>Adjustment Amount</t>
   </si>
   <si>
-    <t>VP/00275/23-24</t>
-  </si>
-  <si>
-    <t>Voucher (AR/AP)</t>
+    <t>ECOM/00205/24-25</t>
+  </si>
+  <si>
+    <t>Retail Sale</t>
+  </si>
+  <si>
+    <t>ECOM/00223/24-25</t>
+  </si>
+  <si>
+    <t>ECOM/00115/24-25</t>
+  </si>
+  <si>
+    <t>TDS/00119/26-27</t>
+  </si>
+  <si>
+    <t>TDS Journal</t>
+  </si>
+  <si>
+    <t>TDS/06868/26-27</t>
   </si>
   <si>
     <t>Reference Site Name</t>
@@ -180,25 +210,25 @@
     </font>
     <font>
       <sz val="9"/>
+      <color rgb="FF171D1E"/>
+      <name val="Courier New"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <color rgb="FF090909"/>
       <name val="Segoe UI"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FF171D1E"/>
+      <color rgb="FF0A0A0A"/>
       <name val="Courier New"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF1F1F1F"/>
-      <name val="Courier New"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF0A0A0A"/>
       <name val="Courier New"/>
       <charset val="134"/>
     </font>
@@ -797,33 +827,30 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1359,8 +1386,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="6"/>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="6"/>
   <cols>
     <col min="2" max="2" width="17.7142857142857" style="1" customWidth="1"/>
     <col min="3" max="3" width="15.7142857142857" style="1" customWidth="1"/>
@@ -1380,7 +1407,7 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
@@ -1409,11 +1436,34 @@
       <c r="E2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="7">
-        <v>46121</v>
+      <c r="F2" s="5">
+        <v>46139</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="5">
+        <v>46139</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1425,8 +1475,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1"/>
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2"/>
   <cols>
     <col min="3" max="3" width="37.2857142857143" style="1" customWidth="1"/>
     <col min="4" max="4" width="29.7142857142857" style="1" customWidth="1"/>
@@ -1444,34 +1494,34 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="J1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="K1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:11">
@@ -1479,28 +1529,57 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2" s="2" t="s">
         <v>26</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>28</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
       </c>
       <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>27</v>
+        <v>1800</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>29</v>
       </c>
       <c r="K2" t="s">
-        <v>28</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1512,8 +1591,8 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="6"/>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="11.4285714285714" style="1" customWidth="1"/>
     <col min="2" max="2" width="7.85714285714286" style="1" customWidth="1"/>
@@ -1529,19 +1608,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E1" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F1" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="G1" t="s">
         <v>6</v>
@@ -1555,13 +1634,30 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D2">
         <v>455352</v>
       </c>
-      <c r="E2" s="7">
-        <v>46121</v>
+      <c r="E2" s="5">
+        <v>46139</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3">
+        <v>455359</v>
+      </c>
+      <c r="E3" s="5">
+        <v>46139</v>
       </c>
     </row>
   </sheetData>
@@ -1573,8 +1669,8 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3"/>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="5"/>
   <cols>
     <col min="3" max="3" width="19.1428571428571" style="1" customWidth="1"/>
     <col min="4" max="4" width="16" style="1" customWidth="1"/>
@@ -1589,28 +1685,28 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C1" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D1" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="E1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="H1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="I1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -1621,27 +1717,97 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="D2" s="3">
-        <v>45094</v>
+        <v>45609</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>450</v>
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="C3" s="4"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="4"/>
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="3">
+        <v>45609</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3">
+        <v>450</v>
+      </c>
     </row>
     <row r="4" spans="1:9">
-      <c r="C4" s="4"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="4"/>
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="3">
+        <v>45609</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="3">
+        <v>46128</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="3">
+        <v>46128</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1661,13 +1827,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Database changes done keeping in mind of parallel execution change
</commit_message>
<xml_diff>
--- a/src/test/resources/Finance/ArVoucher.xlsx
+++ b/src/test/resources/Finance/ArVoucher.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" activeTab="2"/>
+    <workbookView windowWidth="20490" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="DocumentInformation" sheetId="1" r:id="rId1"/>
@@ -1437,7 +1437,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="5">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Ar Voucher stable and Logs & Diagnostics step details missing bug fixing
</commit_message>
<xml_diff>
--- a/src/test/resources/Finance/ArVoucher.xlsx
+++ b/src/test/resources/Finance/ArVoucher.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620"/>
+    <workbookView windowWidth="20490" windowHeight="7620" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="DocumentInformation" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="51">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -177,13 +177,10 @@
     <t>ECOM/00115/24-25</t>
   </si>
   <si>
-    <t>TDS/00119/26-27</t>
+    <t>TDS/06868/26-27</t>
   </si>
   <si>
     <t>TDS Journal</t>
-  </si>
-  <si>
-    <t>TDS/06868/26-27</t>
   </si>
   <si>
     <t>Reference Site Name</t>
@@ -1573,7 +1570,7 @@
         <v>8</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J3" s="8" t="s">
         <v>29</v>
@@ -1669,8 +1666,8 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="5"/>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
     <col min="3" max="3" width="19.1428571428571" style="1" customWidth="1"/>
     <col min="4" max="4" width="16" style="1" customWidth="1"/>
@@ -1786,26 +1783,6 @@
         <v>49</v>
       </c>
       <c r="I5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D6" s="3">
-        <v>46128</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6">
         <v>1</v>
       </c>
     </row>
@@ -1827,7 +1804,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B1" t="s">
         <v>16</v>

</xml_diff>